<commit_message>
Matriz: registrar Irshad (2024) y Alexandre y Balsa (2023)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173jEyEVEUZXo59Qg1UFFEt
</commit_message>
<xml_diff>
--- a/Joaquin/Matriz_Joaquin.xlsx
+++ b/Joaquin/Matriz_Joaquin.xlsx
@@ -416,6 +416,7 @@
   <authors>
     <author>Claude (revisión 07-10-2026)</author>
     <author>Claude (lectura completa 10-10-2026)</author>
+    <author>Claude (10-10-2026)</author>
   </authors>
   <commentList>
     <comment ref="E5" authorId="0" shapeId="0">
@@ -444,6 +445,16 @@
     <comment ref="E9" authorId="0" shapeId="0">
       <text>
         <t>Leído completo (versión aceptada del autor, repositorio NTNU). Datos reales de BN Bank (Noruega), PYMES, 500 767 observaciones, 2021-2023. XGBoost/LGBM/HistGB; AUC 0,94 combinando datos bancarios + crédito + contables (solo bancarios: 0,81-0,85). Clasificación de riesgo del CLIENTE. Limitación para Perumoney: usa datos contables y de crédito de empresas, que una casa de cambio no tiene de personas naturales. Cuartil: pendiente.</t>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="2" shapeId="0">
+      <text>
+        <t>Leído completo; cumple CI1-CI5 y no cae en CE1-CE4. Falta verificar cuartil en Scimago (columna K). Viene de Candidatos_Joaquin.xlsx fila 19.</t>
+      </text>
+    </comment>
+    <comment ref="E11" authorId="2" shapeId="0">
+      <text>
+        <t>Leído completo; cumple CI1-CI5 y no cae en CE1-CE4. Falta verificar cuartil en Scimago (columna K). Viene de Candidatos_Joaquin.xlsx fila 21.</t>
       </text>
     </comment>
   </commentList>
@@ -1336,17 +1347,43 @@
           <t>Joaquín</t>
         </is>
       </c>
-      <c r="D10" s="37" t="n"/>
-      <c r="E10" s="37" t="n"/>
-      <c r="F10" s="37" t="n"/>
-      <c r="G10" s="38" t="n"/>
-      <c r="H10" s="37" t="n"/>
-      <c r="I10" s="37" t="n"/>
-      <c r="J10" s="37" t="n"/>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>Banco o entidad financiera</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>GCF-MLD: Integrated Approach for Money Laundering Detection Using Machine Learning and Graph Network Analysis</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>Irshad, Alkhalifah, Alturise y Khan</t>
+        </is>
+      </c>
+      <c r="G10" s="38" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H10" s="37" t="inlineStr">
+        <is>
+          <t>IEEE Access</t>
+        </is>
+      </c>
+      <c r="I10" s="37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/ACCESS.2024.3510115</t>
+        </is>
+      </c>
+      <c r="J10" s="37" t="inlineStr">
+        <is>
+          <t>Pakistán</t>
+        </is>
+      </c>
       <c r="K10" s="38" t="n"/>
       <c r="L10" s="38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M10" s="39" t="n"/>
@@ -1378,17 +1415,43 @@
           <t>Joaquín</t>
         </is>
       </c>
-      <c r="D11" s="37" t="n"/>
-      <c r="E11" s="37" t="n"/>
-      <c r="F11" s="37" t="n"/>
-      <c r="G11" s="38" t="n"/>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="37" t="n"/>
-      <c r="J11" s="37" t="n"/>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>Banco o entidad financiera</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Incorporating machine learning and a risk-based strategy in an anti-money laundering multiagent system</t>
+        </is>
+      </c>
+      <c r="F11" s="37" t="inlineStr">
+        <is>
+          <t>Alexandre y Balsa</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H11" s="37" t="inlineStr">
+        <is>
+          <t>Expert Systems with Applications</t>
+        </is>
+      </c>
+      <c r="I11" s="37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.eswa.2023.119500</t>
+        </is>
+      </c>
+      <c r="J11" s="37" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
       <c r="K11" s="38" t="n"/>
       <c r="L11" s="38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="M11" s="39" t="n"/>

</xml_diff>